<commit_message>
update : 차트 수정
</commit_message>
<xml_diff>
--- a/Data/SSABT_SETPOINT_TABLE.xlsx
+++ b/Data/SSABT_SETPOINT_TABLE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t>Hz</t>
   </si>
@@ -178,6 +178,78 @@
   </si>
   <si>
     <t>L</t>
+  </si>
+  <si>
+    <t>ㅜ</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>0,280</t>
+  </si>
+  <si>
+    <t>473~5390</t>
+  </si>
+  <si>
+    <t>4730~5390</t>
+  </si>
+  <si>
+    <t>/11</t>
+  </si>
+  <si>
+    <t>/12</t>
+  </si>
+  <si>
+    <t>/13</t>
+  </si>
+  <si>
+    <t>/14</t>
+  </si>
+  <si>
+    <t>/15</t>
+  </si>
+  <si>
+    <t>/16</t>
+  </si>
+  <si>
+    <t>/17</t>
+  </si>
+  <si>
+    <t>/18</t>
+  </si>
+  <si>
+    <t>/19</t>
+  </si>
+  <si>
+    <t>/20</t>
+  </si>
+  <si>
+    <t>0~280</t>
+  </si>
+  <si>
+    <t>3580~3830</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> symbols</t>
+  </si>
+  <si>
+    <t>style</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Symbols</t>
+  </si>
+  <si>
+    <t>Style</t>
+  </si>
+  <si>
+    <t>예비</t>
+  </si>
+  <si>
+    <t>표시 기호</t>
   </si>
 </sst>
 </file>
@@ -538,7 +610,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -657,6 +729,14 @@
         <color theme="4"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -810,7 +890,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -851,6 +931,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1196,7 +1288,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr defaultRowHeight="16.500000"/>
   <cols>
     <col min="3" max="3" width="32.63000107" customWidth="1" outlineLevel="0"/>
@@ -1204,85 +1296,69 @@
     <col min="5" max="5" style="1" width="15.50500011" customWidth="1" outlineLevel="0"/>
     <col min="6" max="7" width="17.62999916" customWidth="1" outlineLevel="0"/>
     <col min="8" max="8" width="14.88000011" customWidth="1" outlineLevel="0"/>
+    <col min="9" max="9" width="25.25499916" customWidth="1" outlineLevel="0"/>
+    <col min="11" max="11" width="23.50499916" customWidth="1" outlineLevel="0"/>
     <col min="12" max="12" width="26.75499916" customWidth="1" outlineLevel="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="G1" s="0" t="s">
+    <row r="2" spans="1:12">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="G2" s="0" t="s">
         <v>48</v>
       </c>
-      <c r="H1" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="I1" s="0" t="s">
+      <c r="H2" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" s="0" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="20.100000" customHeight="1">
-      <c r="A2" s="3" t="s">
+      <c r="J2" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="20.100000" customHeight="1">
+      <c r="A3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="J3" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="L3" s="0" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="20.100000" customHeight="1">
-      <c r="A3" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>0</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="H3" s="3">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2"/>
-      <c r="K3" s="0" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="20.100000" customHeight="1">
+    <row r="4" spans="1:12" ht="20.100000" customHeight="1">
       <c r="A4" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>1</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>17</v>
@@ -1303,15 +1379,19 @@
       <c r="H4" s="3">
         <v>0</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="K4" s="0" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="20.100000" customHeight="1">
+      <c r="I4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="0" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="20.100000" customHeight="1">
       <c r="A5" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>2</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>1</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>17</v>
@@ -1332,12 +1412,19 @@
       <c r="H5" s="3">
         <v>0</v>
       </c>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:11" ht="20.100000" customHeight="1">
+      <c r="I5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="0" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="20.100000" customHeight="1">
       <c r="A6" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>3</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>2</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>17</v>
@@ -1358,328 +1445,392 @@
       <c r="H6" s="3">
         <v>0</v>
       </c>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:11" ht="20.100000" customHeight="1">
-      <c r="A7" s="9">
-        <f>ROW()-ROW($A$2)-1</f>
+      <c r="I6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" ht="20.100000" customHeight="1">
+      <c r="A7" s="3">
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" ht="20.100000" customHeight="1">
+      <c r="A8" s="9">
+        <f>ROW()-ROW($A$3)-1</f>
         <v>4</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="9">
-        <v>4940</v>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H7" s="9">
-        <v>10</v>
-      </c>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:11" ht="20.100000" customHeight="1">
-      <c r="A8" s="9">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>5</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="9">
-        <v>140</v>
-      </c>
-      <c r="F8" s="8"/>
+        <v>4940</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>57</v>
+      </c>
       <c r="G8" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="9">
-        <v>10</v>
-      </c>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="1:11" ht="20.100000" customHeight="1">
+        <v>43</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" ht="20.100000" customHeight="1">
       <c r="A9" s="9">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>6</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>5</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E9" s="9">
-        <v>3720</v>
-      </c>
-      <c r="F9" s="8"/>
+        <v>140</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="G9" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="9">
-        <v>10</v>
-      </c>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="1:11" ht="20.100000" customHeight="1">
+        <v>43</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" ht="20.100000" customHeight="1">
       <c r="A10" s="9">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>7</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>6</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E10" s="9">
-        <v>140</v>
-      </c>
-      <c r="F10" s="8"/>
+        <v>3720</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="G10" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H10" s="9">
-        <v>10</v>
-      </c>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" spans="1:11" ht="20.100000" customHeight="1">
+        <v>43</v>
+      </c>
+      <c r="H10" s="3">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" ht="20.100000" customHeight="1">
       <c r="A11" s="9">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>8</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>7</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E11" s="9">
-        <v>3500</v>
+        <v>140</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H11" s="9">
-        <v>10</v>
-      </c>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="1:11" ht="20.100000" customHeight="1">
+        <v>43</v>
+      </c>
+      <c r="H11" s="3">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+    </row>
+    <row r="12" spans="1:12" ht="20.100000" customHeight="1">
       <c r="A12" s="9">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>9</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>8</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="9">
-        <v>140</v>
+        <v>3500</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H12" s="9">
-        <v>10</v>
-      </c>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:11" ht="20.100000" customHeight="1">
+        <v>43</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+    </row>
+    <row r="13" spans="1:12" ht="20.100000" customHeight="1">
       <c r="A13" s="9">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>10</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>9</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E13" s="9">
-        <v>4040</v>
+        <v>140</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H13" s="9">
+        <v>43</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+    </row>
+    <row r="14" spans="1:12" ht="20.100000" customHeight="1">
+      <c r="A14" s="9">
+        <f>ROW()-ROW($A$3)-1</f>
         <v>10</v>
-      </c>
-      <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:11" ht="20.100000" customHeight="1">
-      <c r="A14" s="9">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>11</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E14" s="9">
-        <v>140</v>
+        <v>4040</v>
       </c>
       <c r="F14" s="8"/>
       <c r="G14" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H14" s="9">
-        <v>10</v>
-      </c>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" spans="1:11" ht="20.100000" customHeight="1">
-      <c r="A15" s="7">
-        <f>ROW()-ROW($A$2)-1</f>
+        <v>43</v>
+      </c>
+      <c r="H14" s="3">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" ht="20.100000" customHeight="1">
+      <c r="A15" s="9">
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>11</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="9">
+        <v>140</v>
+      </c>
+      <c r="F15" s="8"/>
+      <c r="G15" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" ht="20.100000" customHeight="1">
+      <c r="A16" s="7">
+        <f>ROW()-ROW($A$3)-1</f>
         <v>12</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="7">
-        <v>4610</v>
-      </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H15" s="9">
-        <v>10</v>
-      </c>
-      <c r="I15" s="2"/>
-    </row>
-    <row r="16" spans="1:11" ht="20.100000" customHeight="1">
-      <c r="A16" s="7">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>13</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="7">
+        <v>4610</v>
+      </c>
+      <c r="F16" s="6"/>
+      <c r="G16" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" ht="20.100000" customHeight="1">
+      <c r="A17" s="7">
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>13</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="7">
         <v>9750</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H16" s="9">
-        <v>10</v>
-      </c>
-      <c r="I16" s="2"/>
-    </row>
-    <row r="17" spans="1:9" ht="20.100000" customHeight="1">
-      <c r="A17" s="5">
-        <f>ROW()-ROW($A$2)-1</f>
+      <c r="F17" s="6"/>
+      <c r="G17" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+    </row>
+    <row r="18" spans="1:11" ht="20.100000" customHeight="1">
+      <c r="A18" s="5">
+        <f>ROW()-ROW($A$3)-1</f>
         <v>14</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E18" s="5">
         <v>600</v>
       </c>
-      <c r="F17" s="4"/>
-      <c r="G17" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H17" s="9">
-        <v>10</v>
-      </c>
-      <c r="I17" s="2"/>
-    </row>
-    <row r="18" spans="1:9" ht="20.100000" customHeight="1">
-      <c r="A18" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
+      <c r="F18" s="4"/>
+      <c r="G18" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H18" s="3">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+    </row>
+    <row r="19" spans="1:11" ht="20.100000" customHeight="1">
+      <c r="A19" s="3">
+        <f>ROW()-ROW($A$3)-1</f>
         <v>15</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="3">
-        <v>0</v>
-      </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="1:9" ht="20.100000" customHeight="1">
-      <c r="A19" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="3"/>
+        <v>13</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="E19" s="3">
         <v>0</v>
       </c>
@@ -1687,23 +1838,23 @@
       <c r="G19" s="2"/>
       <c r="H19" s="3"/>
       <c r="I19" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="20.100000" customHeight="1">
+        <v>54</v>
+      </c>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A20" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>17</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>16</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>10</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D20" s="3"/>
       <c r="E20" s="3">
         <v>0</v>
       </c>
@@ -1711,161 +1862,195 @@
       <c r="G20" s="2"/>
       <c r="H20" s="3"/>
       <c r="I20" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="20.100000" customHeight="1">
+        <v>46</v>
+      </c>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A21" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>18</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>17</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="E21" s="3">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="3"/>
       <c r="I21" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="20.100000" customHeight="1">
+        <v>51</v>
+      </c>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A22" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>19</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>18</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3">
+        <v>10000</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="3"/>
       <c r="I22" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="20.100000" customHeight="1">
+        <v>46</v>
+      </c>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+    </row>
+    <row r="23" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A23" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>20</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>19</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E23" s="3">
-        <v>620</v>
+        <v>7</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="3"/>
-      <c r="I23" s="2"/>
-    </row>
-    <row r="24" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="I23" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+    </row>
+    <row r="24" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A24" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>21</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>20</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E24" s="3">
-        <v>605</v>
+        <v>620</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="3"/>
-      <c r="I24" s="2"/>
-    </row>
-    <row r="25" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="I24" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A25" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>22</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>21</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E25" s="3">
-        <v>564</v>
+        <v>605</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="2"/>
-    </row>
-    <row r="26" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="I25" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+    </row>
+    <row r="26" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A26" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>23</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>22</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>0</v>
       </c>
       <c r="E26" s="3">
-        <v>580</v>
+        <v>564</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-    </row>
-    <row r="27" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="H26" s="3"/>
+      <c r="I26" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+    </row>
+    <row r="27" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A27" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>24</v>
-      </c>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>23</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3">
+        <v>580</v>
+      </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-    </row>
-    <row r="28" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="I27" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+    </row>
+    <row r="28" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A28" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>25</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>24</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1874,12 +2059,16 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-    </row>
-    <row r="29" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="I28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+    </row>
+    <row r="29" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A29" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>26</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>25</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1888,12 +2077,16 @@
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-    </row>
-    <row r="30" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="I29" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
+    </row>
+    <row r="30" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A30" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>27</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>26</v>
       </c>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1902,12 +2095,16 @@
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-    </row>
-    <row r="31" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="I30" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+    </row>
+    <row r="31" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A31" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>28</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>27</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1916,12 +2113,16 @@
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-    </row>
-    <row r="32" spans="1:9" ht="20.100000" customHeight="1">
+      <c r="I31" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+    </row>
+    <row r="32" spans="1:11" ht="20.100000" customHeight="1">
       <c r="A32" s="3">
-        <f>ROW()-ROW($A$2)-1</f>
-        <v>29</v>
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>28</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1930,10 +2131,34 @@
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-    </row>
-    <row r="33" ht="20.100000" customHeight="1"/>
-    <row r="34" ht="20.100000" customHeight="1"/>
+      <c r="I32" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+    </row>
+    <row r="33" spans="1:11" ht="20.100000" customHeight="1">
+      <c r="A33" s="3">
+        <f>ROW()-ROW($A$3)-1</f>
+        <v>29</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+    </row>
+    <row r="34" spans="1:11" ht="20.100000" customHeight="1">
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+    </row>
     <row r="35" ht="20.100000" customHeight="1"/>
     <row r="36" ht="20.100000" customHeight="1"/>
     <row r="37" ht="20.100000" customHeight="1"/>
@@ -1945,6 +2170,7 @@
     <row r="43" ht="20.100000" customHeight="1"/>
     <row r="44" ht="20.100000" customHeight="1"/>
     <row r="45" ht="20.100000" customHeight="1"/>
+    <row r="46" ht="20.100000" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>

</xml_diff>

<commit_message>
update : plot 수정중
</commit_message>
<xml_diff>
--- a/Data/SSABT_SETPOINT_TABLE.xlsx
+++ b/Data/SSABT_SETPOINT_TABLE.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
   <si>
     <t>Hz</t>
   </si>
@@ -250,6 +250,121 @@
   </si>
   <si>
     <t>표시 기호</t>
+  </si>
+  <si>
+    <t>2710~3170</t>
+  </si>
+  <si>
+    <t>3830~4280</t>
+  </si>
+  <si>
+    <t>0~270</t>
+  </si>
+  <si>
+    <t>260~6000</t>
+  </si>
+  <si>
+    <t>260~5000</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>degree</t>
+  </si>
+  <si>
+    <t>∘</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+      </rPr>
+      <t>∘</t>
+    </r>
+  </si>
+  <si>
+    <t>Sec</t>
+  </si>
+  <si>
+    <t>530~5000</t>
+  </si>
+  <si>
+    <t>0~600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*데이터 테이블 기준표. </t>
+  </si>
+  <si>
+    <t>어드레스</t>
+  </si>
+  <si>
+    <t>타입</t>
+  </si>
+  <si>
+    <t>표서 설명</t>
+  </si>
+  <si>
+    <t>기준 타입</t>
+  </si>
+  <si>
+    <t>기본값</t>
+  </si>
+  <si>
+    <t>정상범위</t>
+  </si>
+  <si>
+    <t>연산 수식</t>
+  </si>
+  <si>
+    <t>설명</t>
+  </si>
+  <si>
+    <t>표시 스타일</t>
+  </si>
+  <si>
+    <t>DefaultRange</t>
+  </si>
+  <si>
+    <t>NormalRange</t>
+  </si>
+  <si>
+    <t>/_10</t>
+  </si>
+  <si>
+    <t>/_11</t>
+  </si>
+  <si>
+    <t>/_12</t>
+  </si>
+  <si>
+    <t>/_13</t>
+  </si>
+  <si>
+    <t>/_14</t>
+  </si>
+  <si>
+    <t>/_15</t>
+  </si>
+  <si>
+    <t>/_16</t>
+  </si>
+  <si>
+    <t>/_17</t>
+  </si>
+  <si>
+    <t>/_18</t>
+  </si>
+  <si>
+    <t>/_19</t>
+  </si>
+  <si>
+    <t>/_20</t>
   </si>
 </sst>
 </file>
@@ -257,7 +372,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11.0"/>
       <name val="맑은 고딕"/>
@@ -394,6 +509,11 @@
       <scheme val="minor"/>
       <color rgb="FF7F7F7F"/>
     </font>
+    <font>
+      <sz val="11.0"/>
+      <name val="맑은 고딕"/>
+      <color theme="1"/>
+    </font>
   </fonts>
   <fills count="36">
     <fill>
@@ -890,7 +1010,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -944,6 +1064,42 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -1288,33 +1444,65 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr defaultRowHeight="16.500000"/>
   <cols>
     <col min="3" max="3" width="32.63000107" customWidth="1" outlineLevel="0"/>
     <col min="4" max="4" style="1" width="10.88000011" customWidth="1" outlineLevel="0"/>
     <col min="5" max="5" style="1" width="15.50500011" customWidth="1" outlineLevel="0"/>
-    <col min="6" max="7" width="17.62999916" customWidth="1" outlineLevel="0"/>
+    <col min="6" max="6" style="1" width="17.62999916" customWidth="1" outlineLevel="0"/>
+    <col min="7" max="7" width="17.62999916" customWidth="1" outlineLevel="0"/>
     <col min="8" max="8" width="14.88000011" customWidth="1" outlineLevel="0"/>
     <col min="9" max="9" width="25.25499916" customWidth="1" outlineLevel="0"/>
     <col min="11" max="11" width="23.50499916" customWidth="1" outlineLevel="0"/>
     <col min="12" max="12" width="26.75499916" customWidth="1" outlineLevel="0"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:12">
+      <c r="B1" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+    </row>
     <row r="2" spans="1:12">
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="A2" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>95</v>
+      </c>
       <c r="G2" s="0" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J2" s="0" t="s">
         <v>75</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="20.100000" customHeight="1">
@@ -1334,7 +1522,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>32</v>
+        <v>100</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>44</v>
@@ -1374,7 +1562,7 @@
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="H4" s="3">
         <v>0</v>
@@ -1407,7 +1595,7 @@
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="H5" s="3">
         <v>0</v>
@@ -1440,7 +1628,7 @@
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="H6" s="3">
         <v>0</v>
@@ -1470,7 +1658,7 @@
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="H7" s="3">
         <v>0</v>
@@ -1498,11 +1686,11 @@
       <c r="E8" s="9">
         <v>4940</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="22" t="s">
         <v>57</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H8" s="3">
         <v>0</v>
@@ -1510,7 +1698,9 @@
       <c r="I8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J8" s="2"/>
+      <c r="J8" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:12" ht="20.100000" customHeight="1">
@@ -1530,19 +1720,21 @@
       <c r="E9" s="9">
         <v>140</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>68</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H9" s="3">
         <v>0</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="J9" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="J9" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:12" ht="20.100000" customHeight="1">
@@ -1562,19 +1754,21 @@
       <c r="E10" s="9">
         <v>3720</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="9" t="s">
         <v>69</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H10" s="3">
         <v>0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="J10" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="J10" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:12" ht="20.100000" customHeight="1">
@@ -1594,9 +1788,11 @@
       <c r="E11" s="9">
         <v>140</v>
       </c>
-      <c r="F11" s="8"/>
+      <c r="F11" s="9" t="s">
+        <v>68</v>
+      </c>
       <c r="G11" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H11" s="3">
         <v>0</v>
@@ -1604,7 +1800,9 @@
       <c r="I11" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J11" s="2"/>
+      <c r="J11" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:12" ht="20.100000" customHeight="1">
@@ -1624,9 +1822,11 @@
       <c r="E12" s="9">
         <v>3500</v>
       </c>
-      <c r="F12" s="8"/>
+      <c r="F12" s="9" t="s">
+        <v>76</v>
+      </c>
       <c r="G12" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H12" s="3">
         <v>0</v>
@@ -1634,7 +1834,9 @@
       <c r="I12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J12" s="2"/>
+      <c r="J12" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:12" ht="20.100000" customHeight="1">
@@ -1654,9 +1856,11 @@
       <c r="E13" s="9">
         <v>140</v>
       </c>
-      <c r="F13" s="8"/>
+      <c r="F13" s="9" t="s">
+        <v>68</v>
+      </c>
       <c r="G13" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H13" s="3">
         <v>0</v>
@@ -1664,7 +1868,9 @@
       <c r="I13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J13" s="2"/>
+      <c r="J13" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:12" ht="20.100000" customHeight="1">
@@ -1684,9 +1890,11 @@
       <c r="E14" s="9">
         <v>4040</v>
       </c>
-      <c r="F14" s="8"/>
+      <c r="F14" s="9" t="s">
+        <v>77</v>
+      </c>
       <c r="G14" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H14" s="3">
         <v>0</v>
@@ -1694,7 +1902,9 @@
       <c r="I14" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J14" s="2"/>
+      <c r="J14" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:12" ht="20.100000" customHeight="1">
@@ -1714,9 +1924,11 @@
       <c r="E15" s="9">
         <v>140</v>
       </c>
-      <c r="F15" s="8"/>
+      <c r="F15" s="9" t="s">
+        <v>78</v>
+      </c>
       <c r="G15" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H15" s="3">
         <v>0</v>
@@ -1724,7 +1936,9 @@
       <c r="I15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J15" s="2"/>
+      <c r="J15" s="21" t="s">
+        <v>81</v>
+      </c>
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:12" ht="20.100000" customHeight="1">
@@ -1744,9 +1958,11 @@
       <c r="E16" s="7">
         <v>4610</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="7" t="s">
+        <v>80</v>
+      </c>
       <c r="G16" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H16" s="3">
         <v>0</v>
@@ -1754,7 +1970,9 @@
       <c r="I16" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J16" s="2"/>
+      <c r="J16" s="21" t="s">
+        <v>82</v>
+      </c>
       <c r="K16" s="2"/>
     </row>
     <row r="17" spans="1:11" ht="20.100000" customHeight="1">
@@ -1774,9 +1992,11 @@
       <c r="E17" s="7">
         <v>9750</v>
       </c>
-      <c r="F17" s="6"/>
+      <c r="F17" s="7" t="s">
+        <v>87</v>
+      </c>
       <c r="G17" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H17" s="3">
         <v>0</v>
@@ -1784,7 +2004,9 @@
       <c r="I17" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J17" s="2"/>
+      <c r="J17" s="21" t="s">
+        <v>82</v>
+      </c>
       <c r="K17" s="2"/>
     </row>
     <row r="18" spans="1:11" ht="20.100000" customHeight="1">
@@ -1804,9 +2026,11 @@
       <c r="E18" s="5">
         <v>600</v>
       </c>
-      <c r="F18" s="4"/>
+      <c r="F18" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="G18" s="9" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="H18" s="3">
         <v>0</v>
@@ -1814,7 +2038,9 @@
       <c r="I18" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J18" s="2"/>
+      <c r="J18" s="21" t="s">
+        <v>85</v>
+      </c>
       <c r="K18" s="2"/>
     </row>
     <row r="19" spans="1:11" ht="20.100000" customHeight="1">
@@ -1834,13 +2060,19 @@
       <c r="E19" s="3">
         <v>0</v>
       </c>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H19" s="3">
+        <v>0</v>
+      </c>
       <c r="I19" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J19" s="2"/>
+      <c r="J19" s="21" t="s">
+        <v>10</v>
+      </c>
       <c r="K19" s="2"/>
     </row>
     <row r="20" spans="1:11" ht="20.100000" customHeight="1">
@@ -1854,17 +2086,25 @@
       <c r="C20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="E20" s="3">
         <v>0</v>
       </c>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H20" s="3">
+        <v>0</v>
+      </c>
       <c r="I20" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="J20" s="2"/>
+      <c r="J20" s="21" t="s">
+        <v>10</v>
+      </c>
       <c r="K20" s="2"/>
     </row>
     <row r="21" spans="1:11" ht="20.100000" customHeight="1">
@@ -1884,13 +2124,19 @@
       <c r="E21" s="3">
         <v>0</v>
       </c>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H21" s="3">
+        <v>0</v>
+      </c>
       <c r="I21" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J21" s="2"/>
+      <c r="J21" s="21" t="s">
+        <v>10</v>
+      </c>
       <c r="K21" s="2"/>
     </row>
     <row r="22" spans="1:11" ht="20.100000" customHeight="1">
@@ -1904,17 +2150,25 @@
       <c r="C22" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="3"/>
+      <c r="D22" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="E22" s="3">
         <v>10000</v>
       </c>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H22" s="3">
+        <v>0</v>
+      </c>
       <c r="I22" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="J22" s="2"/>
+      <c r="J22" s="21" t="s">
+        <v>10</v>
+      </c>
       <c r="K22" s="2"/>
     </row>
     <row r="23" spans="1:11" ht="20.100000" customHeight="1">
@@ -1932,15 +2186,21 @@
         <v>7</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="3"/>
+        <v>42</v>
+      </c>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H23" s="3">
+        <v>0</v>
+      </c>
       <c r="I23" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J23" s="2"/>
+      <c r="J23" s="21" t="s">
+        <v>86</v>
+      </c>
       <c r="K23" s="2"/>
     </row>
     <row r="24" spans="1:11" ht="20.100000" customHeight="1">
@@ -1960,13 +2220,19 @@
       <c r="E24" s="3">
         <v>620</v>
       </c>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H24" s="3">
+        <v>0</v>
+      </c>
       <c r="I24" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J24" s="2"/>
+      <c r="J24" s="21" t="s">
+        <v>0</v>
+      </c>
       <c r="K24" s="2"/>
     </row>
     <row r="25" spans="1:11" ht="20.100000" customHeight="1">
@@ -1986,13 +2252,19 @@
       <c r="E25" s="3">
         <v>605</v>
       </c>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H25" s="3">
+        <v>0</v>
+      </c>
       <c r="I25" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J25" s="2"/>
+      <c r="J25" s="21" t="s">
+        <v>0</v>
+      </c>
       <c r="K25" s="2"/>
     </row>
     <row r="26" spans="1:11" ht="20.100000" customHeight="1">
@@ -2012,13 +2284,19 @@
       <c r="E26" s="3">
         <v>564</v>
       </c>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H26" s="3">
+        <v>0</v>
+      </c>
       <c r="I26" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J26" s="2"/>
+      <c r="J26" s="21" t="s">
+        <v>0</v>
+      </c>
       <c r="K26" s="2"/>
     </row>
     <row r="27" spans="1:11" ht="20.100000" customHeight="1">
@@ -2038,13 +2316,19 @@
       <c r="E27" s="3">
         <v>580</v>
       </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0</v>
+      </c>
       <c r="I27" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="J27" s="2"/>
+      <c r="J27" s="21" t="s">
+        <v>0</v>
+      </c>
       <c r="K27" s="2"/>
     </row>
     <row r="28" spans="1:11" ht="20.100000" customHeight="1">
@@ -2056,9 +2340,13 @@
       <c r="C28" s="2"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H28" s="3">
+        <v>0</v>
+      </c>
       <c r="I28" s="2" t="s">
         <v>54</v>
       </c>
@@ -2074,9 +2362,13 @@
       <c r="C29" s="2"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H29" s="3">
+        <v>0</v>
+      </c>
       <c r="I29" s="2" t="s">
         <v>54</v>
       </c>
@@ -2092,9 +2384,13 @@
       <c r="C30" s="2"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H30" s="3">
+        <v>0</v>
+      </c>
       <c r="I30" s="2" t="s">
         <v>54</v>
       </c>
@@ -2110,9 +2406,13 @@
       <c r="C31" s="2"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H31" s="3">
+        <v>0</v>
+      </c>
       <c r="I31" s="2" t="s">
         <v>54</v>
       </c>
@@ -2128,9 +2428,13 @@
       <c r="C32" s="2"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H32" s="3">
+        <v>0</v>
+      </c>
       <c r="I32" s="2" t="s">
         <v>54</v>
       </c>
@@ -2146,19 +2450,20 @@
       <c r="C33" s="2"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H33" s="3">
+        <v>0</v>
+      </c>
       <c r="I33" s="2" t="s">
         <v>54</v>
       </c>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
     </row>
-    <row r="34" spans="1:11" ht="20.100000" customHeight="1">
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-    </row>
+    <row r="34" ht="20.100000" customHeight="1"/>
     <row r="35" ht="20.100000" customHeight="1"/>
     <row r="36" ht="20.100000" customHeight="1"/>
     <row r="37" ht="20.100000" customHeight="1"/>
@@ -2172,6 +2477,9 @@
     <row r="45" ht="20.100000" customHeight="1"/>
     <row r="46" ht="20.100000" customHeight="1"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:I1"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>